<commit_message>
updated the excel file to use ewerton.mattos@lumonpay.com in the emails columns
</commit_message>
<xml_diff>
--- a/ImportSmallBatchForTest.xlsx
+++ b/ImportSmallBatchForTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ewer\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AB0C467D-D362-4EF2-8D4C-F2CD5FE12ECF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35AD7AE-0AA8-4EAF-ACF6-99E1C43252C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{543EC62A-26F7-482D-96ED-BF73340C8FC4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="218" xr2:uid="{543EC62A-26F7-482D-96ED-BF73340C8FC4}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="181">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="182">
   <si>
     <t>Lead.City</t>
   </si>
@@ -582,6 +582,9 @@
   </si>
   <si>
     <t>Michael kfoury</t>
+  </si>
+  <si>
+    <t>ewerton.mattos@lumonpay.com</t>
   </si>
 </sst>
 </file>
@@ -1059,6 +1062,10 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5C0C2139-B013-4871-B638-12EE72D68F02}">
   <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="8" max="8" width="30.28515625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="25.42578125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:90" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -1353,7 +1360,7 @@
         <v>93</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>94</v>
+        <v>181</v>
       </c>
       <c r="I2" s="7" t="s">
         <v>95</v>
@@ -1439,8 +1446,8 @@
       <c r="AP2" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ2" s="8" t="s">
-        <v>94</v>
+      <c r="AQ2" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR2" s="8"/>
       <c r="AS2" s="8" t="s">
@@ -1591,7 +1598,7 @@
         <v>93</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>115</v>
+        <v>181</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>95</v>
@@ -1679,8 +1686,8 @@
       <c r="AP3" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ3" s="8" t="s">
-        <v>115</v>
+      <c r="AQ3" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR3" s="8"/>
       <c r="AS3" s="8" t="s">
@@ -1830,8 +1837,8 @@
       <c r="G4" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H4" s="8" t="s">
-        <v>127</v>
+      <c r="H4" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>95</v>
@@ -1921,8 +1928,8 @@
       <c r="AP4" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="AQ4" s="8" t="s">
-        <v>127</v>
+      <c r="AQ4" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR4" s="8"/>
       <c r="AS4" s="8" t="s">
@@ -2074,8 +2081,8 @@
       <c r="G5" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H5" s="8" t="s">
-        <v>135</v>
+      <c r="H5" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>95</v>
@@ -2165,8 +2172,8 @@
       <c r="AP5" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ5" s="8" t="s">
-        <v>135</v>
+      <c r="AQ5" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR5" s="8"/>
       <c r="AS5" s="8" t="s">
@@ -2318,8 +2325,8 @@
       <c r="G6" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H6" s="8" t="s">
-        <v>144</v>
+      <c r="H6" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>95</v>
@@ -2407,8 +2414,8 @@
       <c r="AP6" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ6" s="8" t="s">
-        <v>144</v>
+      <c r="AQ6" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR6" s="8"/>
       <c r="AS6" s="8" t="s">
@@ -2556,8 +2563,8 @@
       <c r="G7" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H7" s="8" t="s">
-        <v>155</v>
+      <c r="H7" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>95</v>
@@ -2645,8 +2652,8 @@
       <c r="AP7" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ7" s="8" t="s">
-        <v>155</v>
+      <c r="AQ7" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR7" s="8"/>
       <c r="AS7" s="8" t="s">
@@ -2796,8 +2803,8 @@
       <c r="G8" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H8" s="8" t="s">
-        <v>163</v>
+      <c r="H8" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>95</v>
@@ -2885,8 +2892,8 @@
       <c r="AP8" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="AQ8" s="8" t="s">
-        <v>163</v>
+      <c r="AQ8" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR8" s="8"/>
       <c r="AS8" s="8" t="s">
@@ -3036,8 +3043,8 @@
       <c r="G9" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H9" s="8" t="s">
-        <v>170</v>
+      <c r="H9" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>95</v>
@@ -3125,8 +3132,8 @@
       <c r="AP9" s="8" t="s">
         <v>126</v>
       </c>
-      <c r="AQ9" s="8" t="s">
-        <v>170</v>
+      <c r="AQ9" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR9" s="8"/>
       <c r="AS9" s="8" t="s">
@@ -3276,8 +3283,8 @@
       <c r="G10" s="8" t="s">
         <v>93</v>
       </c>
-      <c r="H10" s="8" t="s">
-        <v>176</v>
+      <c r="H10" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>95</v>
@@ -3363,8 +3370,8 @@
       <c r="AP10" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AQ10" s="8" t="s">
-        <v>176</v>
+      <c r="AQ10" s="10" t="s">
+        <v>181</v>
       </c>
       <c r="AR10" s="8"/>
       <c r="AS10" s="8" t="s">
@@ -3492,8 +3499,24 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="H2" r:id="rId1" display="mailto:phil@totaltmj.co.uk" xr:uid="{86F73E21-A748-4D5C-9204-BFFDAF26CE31}"/>
-    <hyperlink ref="H3" r:id="rId2" display="mailto:freddiemihranian21@gmail.com" xr:uid="{4023CBDE-4A64-4A4C-AB7A-232C95B5C818}"/>
+    <hyperlink ref="H2" r:id="rId1" xr:uid="{86F73E21-A748-4D5C-9204-BFFDAF26CE31}"/>
+    <hyperlink ref="H3" r:id="rId2" xr:uid="{62161F8F-4354-4DAE-AE6D-C2F17016FD76}"/>
+    <hyperlink ref="H4" r:id="rId3" xr:uid="{6C36389A-5CA5-4BF4-9B0C-830E0B9426E9}"/>
+    <hyperlink ref="H5" r:id="rId4" xr:uid="{7D68AD66-E14F-409B-82E9-E837610C84D4}"/>
+    <hyperlink ref="H6" r:id="rId5" xr:uid="{E15C7960-0F09-4EE5-8DAA-BB42EFC10168}"/>
+    <hyperlink ref="H7" r:id="rId6" xr:uid="{E68F7669-1609-42CE-85FD-F1022D62F71B}"/>
+    <hyperlink ref="H8" r:id="rId7" xr:uid="{5D481B19-73FD-4CEA-A453-421E7DAB807C}"/>
+    <hyperlink ref="H9" r:id="rId8" xr:uid="{04D8F575-9D34-4A05-AEA2-C47B78AA45A5}"/>
+    <hyperlink ref="H10" r:id="rId9" xr:uid="{08CEF6CA-B7EF-471E-B57F-ABF5E5DB9402}"/>
+    <hyperlink ref="AQ2" r:id="rId10" xr:uid="{9DBB8470-C14B-4ECD-803E-4D749BC82FF5}"/>
+    <hyperlink ref="AQ3" r:id="rId11" xr:uid="{A8426841-5CCC-48C7-8F67-CB7DD4CAC19D}"/>
+    <hyperlink ref="AQ4" r:id="rId12" xr:uid="{94E1704D-7E62-4DC7-B627-9529ECDBB7CA}"/>
+    <hyperlink ref="AQ5" r:id="rId13" xr:uid="{C87C634F-8A4C-4554-914C-5A3CDBBBB9EC}"/>
+    <hyperlink ref="AQ6" r:id="rId14" xr:uid="{BE893A78-72F9-4F35-8347-5BD977072B14}"/>
+    <hyperlink ref="AQ7" r:id="rId15" xr:uid="{F2EE8C7E-6A65-44B8-B4D7-BDF4FDA80D7B}"/>
+    <hyperlink ref="AQ8" r:id="rId16" xr:uid="{472E99FD-C4CA-4F71-91B2-5760C49DE1F6}"/>
+    <hyperlink ref="AQ9" r:id="rId17" xr:uid="{B6A26499-C444-4167-9365-00486E176E92}"/>
+    <hyperlink ref="AQ10" r:id="rId18" xr:uid="{687310CF-D28C-454F-BDDB-6A539DF8E11B}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
updated emails in the spreadsheet to avoid duplicates
</commit_message>
<xml_diff>
--- a/ImportSmallBatchForTest.xlsx
+++ b/ImportSmallBatchForTest.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ewer\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\currencies-co-uk\FiscalM_AImport\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A35AD7AE-0AA8-4EAF-ACF6-99E1C43252C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78F361C3-BF1E-4B0B-9A9C-1948C952E248}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="218" xr2:uid="{543EC62A-26F7-482D-96ED-BF73340C8FC4}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="667" uniqueCount="190">
   <si>
     <t>Lead.City</t>
   </si>
@@ -585,6 +585,30 @@
   </si>
   <si>
     <t>ewerton.mattos@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos1@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos2@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos3@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos4@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos5@lumonpay.com</t>
+  </si>
+  <si>
+    <t>ewerton.mattos6@lumonpay.com</t>
+  </si>
+  <si>
+    <t>patrick.darling@lumonpay.com</t>
+  </si>
+  <si>
+    <t>Mario.AlexandreCosta@lumonpay.com</t>
   </si>
 </sst>
 </file>
@@ -1063,8 +1087,8 @@
   <dimension ref="A1:CL10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="30.28515625" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="25.42578125" customWidth="1"/>
+    <col min="8" max="8" width="35.85546875" customWidth="1"/>
+    <col min="43" max="43" width="36.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:90" x14ac:dyDescent="0.25">
@@ -1598,7 +1622,7 @@
         <v>93</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="I3" s="8" t="s">
         <v>95</v>
@@ -1687,7 +1711,7 @@
         <v>92</v>
       </c>
       <c r="AQ3" s="10" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="AR3" s="8"/>
       <c r="AS3" s="8" t="s">
@@ -1838,7 +1862,7 @@
         <v>93</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="I4" s="7" t="s">
         <v>95</v>
@@ -1929,7 +1953,7 @@
         <v>126</v>
       </c>
       <c r="AQ4" s="10" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="AR4" s="8"/>
       <c r="AS4" s="8" t="s">
@@ -2082,7 +2106,7 @@
         <v>93</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="I5" s="7" t="s">
         <v>95</v>
@@ -2173,7 +2197,7 @@
         <v>92</v>
       </c>
       <c r="AQ5" s="10" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="AR5" s="8"/>
       <c r="AS5" s="8" t="s">
@@ -2326,7 +2350,7 @@
         <v>93</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I6" s="7" t="s">
         <v>95</v>
@@ -2415,7 +2439,7 @@
         <v>92</v>
       </c>
       <c r="AQ6" s="10" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="AR6" s="8"/>
       <c r="AS6" s="8" t="s">
@@ -2564,7 +2588,7 @@
         <v>93</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="I7" s="7" t="s">
         <v>95</v>
@@ -2653,7 +2677,7 @@
         <v>92</v>
       </c>
       <c r="AQ7" s="10" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="AR7" s="8"/>
       <c r="AS7" s="8" t="s">
@@ -2804,7 +2828,7 @@
         <v>93</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="I8" s="7" t="s">
         <v>95</v>
@@ -2893,7 +2917,7 @@
         <v>126</v>
       </c>
       <c r="AQ8" s="10" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="AR8" s="8"/>
       <c r="AS8" s="8" t="s">
@@ -3044,7 +3068,7 @@
         <v>93</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="I9" s="7" t="s">
         <v>95</v>
@@ -3133,7 +3157,7 @@
         <v>126</v>
       </c>
       <c r="AQ9" s="10" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="AR9" s="8"/>
       <c r="AS9" s="8" t="s">
@@ -3284,7 +3308,7 @@
         <v>93</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="I10" s="7" t="s">
         <v>95</v>
@@ -3371,7 +3395,7 @@
         <v>92</v>
       </c>
       <c r="AQ10" s="10" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="AR10" s="8"/>
       <c r="AS10" s="8" t="s">
@@ -3500,23 +3524,19 @@
   </sheetData>
   <hyperlinks>
     <hyperlink ref="H2" r:id="rId1" xr:uid="{86F73E21-A748-4D5C-9204-BFFDAF26CE31}"/>
-    <hyperlink ref="H3" r:id="rId2" xr:uid="{62161F8F-4354-4DAE-AE6D-C2F17016FD76}"/>
-    <hyperlink ref="H4" r:id="rId3" xr:uid="{6C36389A-5CA5-4BF4-9B0C-830E0B9426E9}"/>
-    <hyperlink ref="H5" r:id="rId4" xr:uid="{7D68AD66-E14F-409B-82E9-E837610C84D4}"/>
-    <hyperlink ref="H6" r:id="rId5" xr:uid="{E15C7960-0F09-4EE5-8DAA-BB42EFC10168}"/>
-    <hyperlink ref="H7" r:id="rId6" xr:uid="{E68F7669-1609-42CE-85FD-F1022D62F71B}"/>
-    <hyperlink ref="H8" r:id="rId7" xr:uid="{5D481B19-73FD-4CEA-A453-421E7DAB807C}"/>
-    <hyperlink ref="H9" r:id="rId8" xr:uid="{04D8F575-9D34-4A05-AEA2-C47B78AA45A5}"/>
-    <hyperlink ref="H10" r:id="rId9" xr:uid="{08CEF6CA-B7EF-471E-B57F-ABF5E5DB9402}"/>
-    <hyperlink ref="AQ2" r:id="rId10" xr:uid="{9DBB8470-C14B-4ECD-803E-4D749BC82FF5}"/>
-    <hyperlink ref="AQ3" r:id="rId11" xr:uid="{A8426841-5CCC-48C7-8F67-CB7DD4CAC19D}"/>
-    <hyperlink ref="AQ4" r:id="rId12" xr:uid="{94E1704D-7E62-4DC7-B627-9529ECDBB7CA}"/>
-    <hyperlink ref="AQ5" r:id="rId13" xr:uid="{C87C634F-8A4C-4554-914C-5A3CDBBBB9EC}"/>
-    <hyperlink ref="AQ6" r:id="rId14" xr:uid="{BE893A78-72F9-4F35-8347-5BD977072B14}"/>
-    <hyperlink ref="AQ7" r:id="rId15" xr:uid="{F2EE8C7E-6A65-44B8-B4D7-BDF4FDA80D7B}"/>
-    <hyperlink ref="AQ8" r:id="rId16" xr:uid="{472E99FD-C4CA-4F71-91B2-5760C49DE1F6}"/>
-    <hyperlink ref="AQ9" r:id="rId17" xr:uid="{B6A26499-C444-4167-9365-00486E176E92}"/>
-    <hyperlink ref="AQ10" r:id="rId18" xr:uid="{687310CF-D28C-454F-BDDB-6A539DF8E11B}"/>
+    <hyperlink ref="H5" r:id="rId2" xr:uid="{7D68AD66-E14F-409B-82E9-E837610C84D4}"/>
+    <hyperlink ref="H6" r:id="rId3" xr:uid="{E15C7960-0F09-4EE5-8DAA-BB42EFC10168}"/>
+    <hyperlink ref="H7" r:id="rId4" xr:uid="{E68F7669-1609-42CE-85FD-F1022D62F71B}"/>
+    <hyperlink ref="H8" r:id="rId5" xr:uid="{5D481B19-73FD-4CEA-A453-421E7DAB807C}"/>
+    <hyperlink ref="H9" r:id="rId6" xr:uid="{04D8F575-9D34-4A05-AEA2-C47B78AA45A5}"/>
+    <hyperlink ref="H10" r:id="rId7" xr:uid="{08CEF6CA-B7EF-471E-B57F-ABF5E5DB9402}"/>
+    <hyperlink ref="AQ2" r:id="rId8" xr:uid="{B4CE8F2D-D18B-4EB7-897A-4740F8DC616D}"/>
+    <hyperlink ref="AQ5" r:id="rId9" xr:uid="{80CC2C5C-BC92-4022-AB8F-922EF76E3DDE}"/>
+    <hyperlink ref="AQ6" r:id="rId10" xr:uid="{16E0480F-0BF9-4D2D-B574-8B247542FF87}"/>
+    <hyperlink ref="AQ7" r:id="rId11" xr:uid="{165845D5-009D-4CA7-95D8-9FA663E9EFCC}"/>
+    <hyperlink ref="AQ8" r:id="rId12" xr:uid="{5CD62BCD-ABC0-4405-88F2-0D54EFDFCA30}"/>
+    <hyperlink ref="AQ9" r:id="rId13" xr:uid="{D01BAED2-63ED-41E1-96F8-AC8DC0210CA6}"/>
+    <hyperlink ref="AQ10" r:id="rId14" xr:uid="{90EB5984-F7BA-4DD6-83B0-A0B3C702A663}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>